<commit_message>
fix: template import theo hàng ngang (header 1 dòng, mỗi SP 1 dòng)
Không liệt kê field dọc; 3 cột product_name | retail_price | inventory.
</commit_message>
<xml_diff>
--- a/import-templates/product-import-template.xlsx
+++ b/import-templates/product-import-template.xlsx
@@ -12,27 +12,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
   <si>
     <t>Vinameals — Simple product import</t>
   </si>
   <si>
-    <t>Only 3 columns required on the Products sheet:</t>
-  </si>
-  <si>
-    <t>product_name | retail_price | inventory</t>
-  </si>
-  <si>
-    <t>Each row creates one product with auto ID, handle, and SKU.</t>
-  </si>
-  <si>
-    <t>No category → product only appears under Shop all until you assign a category.</t>
-  </si>
-  <si>
-    <t>Images and video: upload later in Admin → Products.</t>
-  </si>
-  <si>
-    <t>Optional columns (if present): sale_price, cost_price, sku, short_description, status</t>
+    <t>How to fill</t>
+  </si>
+  <si>
+    <t>Use the Products sheet. Headers are on ONE horizontal row. Each product is ONE horizontal data row under the headers.</t>
+  </si>
+  <si>
+    <t>Required columns (left → right on Products sheet)</t>
   </si>
   <si>
     <t>product_name</t>
@@ -44,10 +35,28 @@
     <t>inventory</t>
   </si>
   <si>
+    <t>Tên sản phẩm</t>
+  </si>
+  <si>
+    <t>Giá bán (USD)</t>
+  </si>
+  <si>
+    <t>Số lượng tồn</t>
+  </si>
+  <si>
+    <t>Example (same layout as Products sheet)</t>
+  </si>
+  <si>
     <t>Tropical Mango Slices</t>
   </si>
   <si>
     <t>Garden Veggie Dumplings</t>
+  </si>
+  <si>
+    <t>Do NOT list fields vertically (one field per row). Always use columns across the top, products down the rows.</t>
+  </si>
+  <si>
+    <t>Auto-created: product ID, handle, slug, SKU. No category → only Shop all. Images later in Admin.</t>
   </si>
   <si>
     <t>Golden Chili Crisp</t>
@@ -57,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -67,18 +76,41 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF075B40"/>
       <sz val="16"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFB42318"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDFF7E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B7A55"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -93,10 +125,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,45 +482,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C11" s="6" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>8.99</v>
+      </c>
+      <c r="C12">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>12.99</v>
+      </c>
+      <c r="C13">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A17:C17"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -485,27 +605,27 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>9</v>
+    <row r="1" ht="22" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="B2" s="10">
         <v>8.99</v>
       </c>
       <c r="C2">
@@ -514,9 +634,9 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
+        <v>12</v>
+      </c>
+      <c r="B3" s="10">
         <v>12.99</v>
       </c>
       <c r="C3">
@@ -525,9 +645,9 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="10">
         <v>10.5</v>
       </c>
       <c r="C4">
@@ -535,6 +655,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>